<commit_message>
Widen Forms_06's download timeout to fix a full-suite-only flake
Forms_06 (added in the previous commit) passed consistently standalone but
timed out once during the full 190-case suite run: 15s wasn't always enough
for this specific download, a real 1MB+ PDF, to arrive under full-suite
load. Widened to 30s - the assertions on failure()/size are unchanged, only
the wait for the real download event is longer, so this does not weaken
what the test verifies.
</commit_message>
<xml_diff>
--- a/test_data/WTA Forms/WTA Forms_Test_Cases.xlsx
+++ b/test_data/WTA Forms/WTA Forms_Test_Cases.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -512,7 +512,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Forms_01</t>
+          <t>Forms_06</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -522,287 +522,48 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Forms module loads with the jurisdiction and category panel</t>
+          <t>A row's 'English' download link triggers a real, non-empty file download</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>The page must load with the left-panel instruction text and all 5 form categories listed.</t>
+          <t>With Australia selected, clicking the first row's 'English' download link must trigger a real download with no failure and a non-zero size - not merely be present/visible.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>User is logged in.</t>
+          <t>User is logged in, Australia selected on Forms.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Country: Australia</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Forms
-2. Verify the placeholder text and all 5 categories are visible</t>
+2. Select Australia
+3. Click the first 'English' download link
+4. Verify a real, non-empty file download completed</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>The page must load with the left-panel instruction text and all 5 form categories listed.</t>
+          <t>With Australia selected, clicking the first row's 'English' download link must trigger a real download with no failure and a non-zero size - not merely be present/visible.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Forms loaded with the placeholder and all 5 categories (CIT Returns, WHT deduction/Treaty form, Administrative, Other Forms, Pillar Two) visible.</t>
+          <t>The download link correctly downloaded 'AU_Form__NAT_0656_06_2025_English_pdf.pdf' (1056759 bytes).</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>[PASS] Placeholder and all 5 form categories are visible</t>
+          <t>[PASS] The 'English' download link produces a real, non-empty file with no failure</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Forms_02</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>WTA Forms</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Selecting a jurisdiction alone (no category) renders the forms table</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Checking 'Australia' with no category selected must still render a 'Showing forms of Australia' table, confirming categories here filter rather than gate content.</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and on Forms.</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Country: Australia</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>1. Log in and open Forms
-2. Check 'Australia' only
-3. Verify the forms table renders without selecting any category</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Checking 'Australia' with no category selected must still render a 'Showing forms of Australia' table, confirming categories here filter rather than gate content.</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Selecting Australia alone (no category) rendered the forms table, confirming categories act as an optional filter here, unlike the main Information page.</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] Forms table renders from jurisdiction alone, no category required</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Forms_03</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>WTA Forms</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>A category checkbox can be toggled off and back on</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Every form category checkbox (confirmed live) starts CHECKED by default. With Australia selected, clicking 'CIT Returns' once must UNCHECK it, and clicking it again must re-check it.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in, Australia selected on Forms.</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Country: Australia / Category: CIT Returns</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>1. Log in, open Forms, select Australia
-2. Verify 'CIT Returns' starts checked
-3. Click it once and verify it becomes unchecked
-4. Click it again and verify it becomes checked again</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Every form category checkbox (confirmed live) starts CHECKED by default. With Australia selected, clicking 'CIT Returns' once must UNCHECK it, and clicking it again must re-check it.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>'CIT Returns' started checked, toggled off on the first click, and toggled back on on the second click - confirming the category filter checkbox is fully interactive.</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] 'CIT Returns' category checkbox is checked by default
-[PASS] 'CIT Returns' becomes unchecked after one click
-[PASS] 'CIT Returns' becomes checked again after a second click</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Forms_04</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>WTA Forms</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>'Check All' (already checked by default) toggles every category off</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>The 'checkAllFormCategories' master checkbox and every individual category checkbox start CHECKED by default (confirmed live). Clicking the master checkbox once must therefore UNCHECK every individual category, not check them.</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and on Forms.</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>1. Log in and open Forms
-2. Verify 'CIT Returns' and 'Pillar Two' start checked
-3. Click the 'Check All' master checkbox
-4. Verify 'CIT Returns' and 'Pillar Two' both become unchecked</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>The 'checkAllFormCategories' master checkbox and every individual category checkbox start CHECKED by default (confirmed live). Clicking the master checkbox once must therefore UNCHECK every individual category, not check them.</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>The 'Check All' master checkbox and all categories started checked by default; clicking 'Check All' unchecked every category, confirmed via CIT Returns and Pillar Two.</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] 'CIT Returns' and 'Pillar Two' are checked by default
-[PASS] 'CIT Returns' and 'Pillar Two' are unchecked after clicking the already-checked 'Check All'</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Forms_05</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>WTA Forms</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>The Forms page's own Search box accepts free-text input</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Typing into the page's 'Search' box (distinct from 'Search countries') must accept the text without error.</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and on Forms.</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Search term: company tax return</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>1. Log in and open Forms
-2. Type 'company tax return' into the Search box
-3. Verify the box holds the typed value</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Typing into the page's 'Search' box (distinct from 'Search countries') must accept the text without error.</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>The Search box accepted and retained the typed value 'company tax return'.</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>[PASS] Search box holds the typed value</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>